<commit_message>
- Small changes to Dashboard/Streamlit_Dashboard.py
</commit_message>
<xml_diff>
--- a/notebooks/Dashboard/chart_info.xlsx
+++ b/notebooks/Dashboard/chart_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ma1066\Documents\Code\peexcel\notebooks\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87AA554E-E334-4BB3-8DED-079BD1D4D8DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62ECC837-5829-4F19-AF29-300610FE0187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1065" yWindow="2565" windowWidth="17400" windowHeight="16335" xr2:uid="{8863A408-E089-4CD0-AD5E-01FA994FFACD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{8863A408-E089-4CD0-AD5E-01FA994FFACD}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="238">
   <si>
     <t>domain</t>
   </si>
@@ -138,12 +138,6 @@
     <t>diagram</t>
   </si>
   <si>
-    <t>x-axis</t>
-  </si>
-  <si>
-    <t>y-axis</t>
-  </si>
-  <si>
     <t>Primärenergiebedarf</t>
   </si>
   <si>
@@ -183,21 +177,9 @@
     <t>gwp_ee_detail</t>
   </si>
   <si>
-    <t>GWP_lc_total</t>
-  </si>
-  <si>
-    <t>Balance Variable</t>
-  </si>
-  <si>
     <t>district_gwp_ee</t>
   </si>
   <si>
-    <t>GWP_ee_total_biogenic</t>
-  </si>
-  <si>
-    <t>GWP_oe_grid_feedin</t>
-  </si>
-  <si>
     <t>multi_chart</t>
   </si>
   <si>
@@ -252,30 +234,9 @@
     <t>Eev_ext_charge</t>
   </si>
   <si>
-    <t>GWP_ee_lc_mob</t>
-  </si>
-  <si>
     <t>GWP_ee_solarthermal</t>
   </si>
   <si>
-    <t>GWP_ee_total_construction_biogenic</t>
-  </si>
-  <si>
-    <t>GWP_lc_EE_total</t>
-  </si>
-  <si>
-    <t>GWP_lc_OE_total</t>
-  </si>
-  <si>
-    <t>GWP_oe_mob_ev_export</t>
-  </si>
-  <si>
-    <t>GWP_oe_mob_ev</t>
-  </si>
-  <si>
-    <t>GWP_oe_mob_fossile</t>
-  </si>
-  <si>
     <t>GWP_ee_wall</t>
   </si>
   <si>
@@ -297,33 +258,6 @@
     <t>GWP_ee_ceiling</t>
   </si>
   <si>
-    <t>GWP_emInt_grid</t>
-  </si>
-  <si>
-    <t>GWP_emInt_flex</t>
-  </si>
-  <si>
-    <t>GWP_oe_district_heating</t>
-  </si>
-  <si>
-    <t>GWP_oe_other</t>
-  </si>
-  <si>
-    <t>GWP_ee_total_construction</t>
-  </si>
-  <si>
-    <t>GWP_ee_total_TES</t>
-  </si>
-  <si>
-    <t>GWP_oe_building</t>
-  </si>
-  <si>
-    <t>GWP_ee_mob_fossile</t>
-  </si>
-  <si>
-    <t>GWP_ee_mob_ev</t>
-  </si>
-  <si>
     <t>Nutzerstrom</t>
   </si>
   <si>
@@ -435,36 +369,9 @@
     <t>E-Car Ladung Außerhalb des Quartiers</t>
   </si>
   <si>
-    <t>Errichtung Mobilität</t>
-  </si>
-  <si>
     <t>THG LZ Solarthermie</t>
   </si>
   <si>
-    <t>THG Graue Energie LZ Baulich Biogen</t>
-  </si>
-  <si>
-    <t>EE THG-Emissionen 2025-2075</t>
-  </si>
-  <si>
-    <t>OE THG-Emissionen 2025-2075</t>
-  </si>
-  <si>
-    <t>GWP MIV Export (Anderer Verkehr)</t>
-  </si>
-  <si>
-    <t>GWP MIV elektrisch INSGESAMTE LADUNG</t>
-  </si>
-  <si>
-    <t>GWP MIV fossil</t>
-  </si>
-  <si>
-    <t>Betrieb Netzeinspeisung</t>
-  </si>
-  <si>
-    <t>THG-Emissionen 2025-2075</t>
-  </si>
-  <si>
     <t>THG LZ Außenwand</t>
   </si>
   <si>
@@ -486,36 +393,6 @@
     <t>THG LZ Geschossdecke</t>
   </si>
   <si>
-    <t>Emissions-Intensität Netzstrombezug</t>
-  </si>
-  <si>
-    <t>Emissions-Intensität Flexibler Netzbezug</t>
-  </si>
-  <si>
-    <t>Betrieb HKLS Fernwärme</t>
-  </si>
-  <si>
-    <t>Betrieb HKLS Sonstige</t>
-  </si>
-  <si>
-    <t>THG Graue Energie LZ Baulich</t>
-  </si>
-  <si>
-    <t>THG Graue Energie LZ TGA</t>
-  </si>
-  <si>
-    <t>Errichtung Mobilität fossil</t>
-  </si>
-  <si>
-    <t>Errichtung Mobilität Elektrisch</t>
-  </si>
-  <si>
-    <t>THG Graue Energie LZ Biogen</t>
-  </si>
-  <si>
-    <t>Betrieb Gebäude</t>
-  </si>
-  <si>
     <t>#7e1141</t>
   </si>
   <si>
@@ -609,48 +486,12 @@
     <t>#faf2bf</t>
   </si>
   <si>
-    <t>#B87500</t>
-  </si>
-  <si>
-    <t>#eb4197</t>
-  </si>
-  <si>
-    <t>#33abba</t>
-  </si>
-  <si>
-    <t>#bbce00</t>
-  </si>
-  <si>
-    <t>#E9FF0D</t>
-  </si>
-  <si>
-    <t>#F9FFC2</t>
-  </si>
-  <si>
-    <t>#60b564</t>
-  </si>
-  <si>
-    <t>#d7eff3</t>
-  </si>
-  <si>
-    <t>#b0dfe5</t>
-  </si>
-  <si>
-    <t>#eeff49</t>
-  </si>
-  <si>
     <t>/</t>
   </si>
   <si>
     <t>x</t>
   </si>
   <si>
-    <t>+</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>final_energy_balance</t>
   </si>
   <si>
@@ -663,12 +504,6 @@
     <t>WW E-Stab</t>
   </si>
   <si>
-    <t>embodied_emissions</t>
-  </si>
-  <si>
-    <t>operational_emissions</t>
-  </si>
-  <si>
     <t>tab_name</t>
   </si>
   <si>
@@ -678,7 +513,247 @@
     <t>title</t>
   </si>
   <si>
-    <t>#8d9b00</t>
+    <t>GWP_ee_floor</t>
+  </si>
+  <si>
+    <t>GWP_ee_terrace</t>
+  </si>
+  <si>
+    <t>GWP_ee_basement_ceiling</t>
+  </si>
+  <si>
+    <t>GWP_ee_ceil_to_air</t>
+  </si>
+  <si>
+    <t>GWP_ee_wall_earth_contacted</t>
+  </si>
+  <si>
+    <t>GWP_ee_internal_wall_load</t>
+  </si>
+  <si>
+    <t>GWP_ee_internal_wall_nonload</t>
+  </si>
+  <si>
+    <t>GWP_ee_ceiling_topfloor</t>
+  </si>
+  <si>
+    <t>GWP_ee_wall_ec_unheated</t>
+  </si>
+  <si>
+    <t>GWP_ee_basement_floor_unheated</t>
+  </si>
+  <si>
+    <t>GWP_ee_columns</t>
+  </si>
+  <si>
+    <t>GWP_ee_internal_wall_unheated</t>
+  </si>
+  <si>
+    <t>GWP_ee_unheated_horizontal</t>
+  </si>
+  <si>
+    <t>GWP_ee_balconies</t>
+  </si>
+  <si>
+    <t>GWP_ee_garage_horizontal</t>
+  </si>
+  <si>
+    <t>GWP_ee_garage_columns</t>
+  </si>
+  <si>
+    <t>GWP_ee_other_1</t>
+  </si>
+  <si>
+    <t>GWP_ee_other_2</t>
+  </si>
+  <si>
+    <t>GWP_ee_other_3</t>
+  </si>
+  <si>
+    <t>GWP_ee_PV</t>
+  </si>
+  <si>
+    <t>GWP_ee_boreholes</t>
+  </si>
+  <si>
+    <t>GWP_ee_ahu_1</t>
+  </si>
+  <si>
+    <t>GWP_ee_ahu_2</t>
+  </si>
+  <si>
+    <t>GWP_ee_buffer_storage</t>
+  </si>
+  <si>
+    <t>GWP_ee_BESS</t>
+  </si>
+  <si>
+    <t>GWP_ee_energy_1</t>
+  </si>
+  <si>
+    <t>GWP_ee_energy_2</t>
+  </si>
+  <si>
+    <t>THG LZ Erdb. Fußboden beheizt</t>
+  </si>
+  <si>
+    <t>THG LZ Terasse</t>
+  </si>
+  <si>
+    <t>THG LZ Kellerdecke</t>
+  </si>
+  <si>
+    <t>THG LZ Außendecke gg. Außenluft</t>
+  </si>
+  <si>
+    <t>THG LZ Erdb. Wand beheizt</t>
+  </si>
+  <si>
+    <t>THG LZ Innenwand tragend</t>
+  </si>
+  <si>
+    <t>THG LZ Innenwand nicht tragend</t>
+  </si>
+  <si>
+    <t>THG LZ Oberste Geschoßdecke</t>
+  </si>
+  <si>
+    <t>THG LZ Erdb. Wand Keller</t>
+  </si>
+  <si>
+    <t>THG LZ Erdb. Fußboden unbeheizt</t>
+  </si>
+  <si>
+    <t>THG LZ Stützen</t>
+  </si>
+  <si>
+    <t>THG LZ Innenwand unbeheizt</t>
+  </si>
+  <si>
+    <t>THG LZ Zwischendecke unbeheizt / Keller / TG</t>
+  </si>
+  <si>
+    <t>THG LZ Balkone</t>
+  </si>
+  <si>
+    <t>THG LZ Garage Decken</t>
+  </si>
+  <si>
+    <t>THG LZ Garage Stützen</t>
+  </si>
+  <si>
+    <t>THG LZ Sonstige 2</t>
+  </si>
+  <si>
+    <t>THG LZ Sonstige 3</t>
+  </si>
+  <si>
+    <t>THG LZ PV-Anlage</t>
+  </si>
+  <si>
+    <t>THG LZ Erdwärmesonden</t>
+  </si>
+  <si>
+    <t>THG LZ Lüftungsanlage 1</t>
+  </si>
+  <si>
+    <t>THG LZ Lüftungsanlage 2</t>
+  </si>
+  <si>
+    <t>THG LZ Pufferspeicher</t>
+  </si>
+  <si>
+    <t>THG LZ E-Batterie</t>
+  </si>
+  <si>
+    <t>THG LZ Energiesystem 1</t>
+  </si>
+  <si>
+    <t>THG LZ Energiesystem 2</t>
+  </si>
+  <si>
+    <t>THG LZ Sonstige 1</t>
+  </si>
+  <si>
+    <t>Baulich</t>
+  </si>
+  <si>
+    <t>Betrieblich</t>
+  </si>
+  <si>
+    <t>Baulich kompensation</t>
+  </si>
+  <si>
+    <t>Betrieblich kompensation</t>
+  </si>
+  <si>
+    <t>Optionen für destination</t>
+  </si>
+  <si>
+    <t>#f9c0dd</t>
+  </si>
+  <si>
+    <t>#9fd3a2</t>
+  </si>
+  <si>
+    <t>#418e48</t>
+  </si>
+  <si>
+    <t>#2c5e2f</t>
+  </si>
+  <si>
+    <t>#ffc560</t>
+  </si>
+  <si>
+    <t>#f281bb</t>
+  </si>
+  <si>
+    <t>#a6a6a6</t>
+  </si>
+  <si>
+    <t>#d9d9d9</t>
+  </si>
+  <si>
+    <t>#3d5b38</t>
+  </si>
+  <si>
+    <t>#950f53</t>
+  </si>
+  <si>
+    <t>#418e46</t>
+  </si>
+  <si>
+    <t>#595959</t>
+  </si>
+  <si>
+    <t>#bfbfbf</t>
+  </si>
+  <si>
+    <t>#ffd895</t>
+  </si>
+  <si>
+    <t>#000000</t>
+  </si>
+  <si>
+    <t>#88cfda</t>
+  </si>
+  <si>
+    <t>#7f7f7f</t>
+  </si>
+  <si>
+    <t>#e9ff0d</t>
+  </si>
+  <si>
+    <t>#e1320f</t>
+  </si>
+  <si>
+    <t>#88ced8</t>
+  </si>
+  <si>
+    <t>#c47d00</t>
+  </si>
+  <si>
+    <t>#b87500</t>
   </si>
 </sst>
 </file>
@@ -1053,15 +1128,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7A2313-314F-4C5D-9E95-F307104932AD}">
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1081,12 +1156,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -1095,15 +1170,18 @@
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="I2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
@@ -1112,15 +1190,18 @@
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -1129,15 +1210,18 @@
         <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+      <c r="I4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
@@ -1146,15 +1230,18 @@
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+      <c r="I5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -1163,15 +1250,18 @@
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+      <c r="I6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1180,15 +1270,18 @@
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+      <c r="I7" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
         <v>13</v>
@@ -1197,15 +1290,18 @@
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+      <c r="I8" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
@@ -1214,15 +1310,15 @@
         <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
@@ -1231,18 +1327,18 @@
         <v>16</v>
       </c>
       <c r="E10" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
       <c r="F10" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
@@ -1251,18 +1347,18 @@
         <v>17</v>
       </c>
       <c r="E11" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
       <c r="F11" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
@@ -1271,15 +1367,15 @@
         <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
         <v>19</v>
@@ -1288,15 +1384,15 @@
         <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
@@ -1305,18 +1401,18 @@
         <v>17</v>
       </c>
       <c r="E14" t="s">
-        <v>169</v>
+        <v>128</v>
       </c>
       <c r="F14" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
         <v>22</v>
@@ -1325,18 +1421,18 @@
         <v>17</v>
       </c>
       <c r="E15" t="s">
-        <v>170</v>
+        <v>129</v>
       </c>
       <c r="F15" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
         <v>24</v>
@@ -1345,7 +1441,7 @@
         <v>16</v>
       </c>
       <c r="E16" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1353,7 +1449,7 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="C17" t="s">
         <v>25</v>
@@ -1362,7 +1458,7 @@
         <v>16</v>
       </c>
       <c r="E17" t="s">
-        <v>171</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1370,7 +1466,7 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="C18" t="s">
         <v>26</v>
@@ -1379,7 +1475,7 @@
         <v>16</v>
       </c>
       <c r="E18" t="s">
-        <v>172</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1387,7 +1483,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
         <v>27</v>
@@ -1396,7 +1492,7 @@
         <v>16</v>
       </c>
       <c r="E19" t="s">
-        <v>173</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1404,7 +1500,7 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>112</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
         <v>28</v>
@@ -1413,7 +1509,7 @@
         <v>17</v>
       </c>
       <c r="E20" t="s">
-        <v>174</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1421,7 +1517,7 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
         <v>29</v>
@@ -1430,7 +1526,7 @@
         <v>17</v>
       </c>
       <c r="E21" t="s">
-        <v>175</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1438,7 +1534,7 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="C22" t="s">
         <v>30</v>
@@ -1447,967 +1543,914 @@
         <v>17</v>
       </c>
       <c r="E22" t="s">
-        <v>176</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B23" t="s">
-        <v>115</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
         <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>177</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B24" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="C24" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D24" t="s">
         <v>16</v>
       </c>
       <c r="E24" t="s">
-        <v>178</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B25" t="s">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D25" t="s">
         <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>179</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B26" t="s">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="C26" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D26" t="s">
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>180</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B27" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D27" t="s">
         <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>176</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B28" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B29" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="C29" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D29" t="s">
         <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>174</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B30" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="C30" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D30" t="s">
         <v>17</v>
       </c>
       <c r="E30" t="s">
-        <v>182</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>206</v>
+        <v>153</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
         <v>17</v>
       </c>
       <c r="E31" t="s">
-        <v>183</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B32" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="C32" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
       </c>
       <c r="E32" t="s">
-        <v>184</v>
+        <v>143</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B33" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="C33" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
       </c>
       <c r="E33" t="s">
-        <v>185</v>
+        <v>144</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B34" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="C34" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D34" t="s">
         <v>17</v>
       </c>
       <c r="E34" t="s">
-        <v>167</v>
+        <v>126</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B35" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="C35" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
       </c>
       <c r="E35" t="s">
-        <v>186</v>
+        <v>145</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B36" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="C36" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D36" t="s">
         <v>17</v>
       </c>
       <c r="E36" t="s">
-        <v>187</v>
+        <v>146</v>
       </c>
       <c r="F36" t="s">
-        <v>199</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B37" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C37" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D37" t="s">
         <v>17</v>
       </c>
       <c r="E37" t="s">
-        <v>188</v>
+        <v>147</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B38" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
       <c r="C38" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
       </c>
       <c r="E38" t="s">
-        <v>183</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B39" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="C39" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D39" t="s">
         <v>17</v>
       </c>
       <c r="E39" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="C40" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D40" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E40" t="s">
-        <v>189</v>
-      </c>
-      <c r="F40" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B41" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="C41" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D41" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E41" t="s">
-        <v>190</v>
+        <v>217</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="C42" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D42" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E42" t="s">
-        <v>191</v>
+        <v>217</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>134</v>
+        <v>184</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>157</v>
       </c>
       <c r="D43" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E43" t="s">
-        <v>191</v>
+        <v>218</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="C44" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D44" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E44" t="s">
-        <v>192</v>
+        <v>219</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>158</v>
       </c>
       <c r="D45" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E45" t="s">
-        <v>193</v>
+        <v>220</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>137</v>
+        <v>186</v>
       </c>
       <c r="C46" t="s">
-        <v>76</v>
+        <v>159</v>
       </c>
       <c r="D46" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E46" t="s">
-        <v>194</v>
-      </c>
-      <c r="F46" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B47" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="D47" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E47" t="s">
-        <v>189</v>
-      </c>
-      <c r="F47" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B48" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="C48" t="s">
-        <v>51</v>
+        <v>160</v>
       </c>
       <c r="D48" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E48" t="s">
-        <v>195</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B49" t="s">
-        <v>140</v>
+        <v>188</v>
       </c>
       <c r="C49" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
       <c r="D49" t="s">
-        <v>48</v>
+        <v>211</v>
       </c>
       <c r="E49" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B50" t="s">
-        <v>141</v>
+        <v>189</v>
       </c>
       <c r="C50" t="s">
-        <v>78</v>
+        <v>162</v>
       </c>
       <c r="D50" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E50" t="s">
-        <v>196</v>
-      </c>
-      <c r="F50" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B51" t="s">
-        <v>142</v>
+        <v>190</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>163</v>
       </c>
       <c r="D51" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E51" t="s">
-        <v>196</v>
+        <v>223</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B52" t="s">
-        <v>143</v>
+        <v>191</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
+        <v>164</v>
       </c>
       <c r="D52" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E52" t="s">
-        <v>196</v>
+        <v>224</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B53" t="s">
-        <v>144</v>
+        <v>192</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
+        <v>165</v>
       </c>
       <c r="D53" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E53" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B54" t="s">
-        <v>145</v>
+        <v>193</v>
       </c>
       <c r="C54" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="D54" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E54" t="s">
-        <v>196</v>
+        <v>226</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B55" t="s">
-        <v>146</v>
+        <v>194</v>
       </c>
       <c r="C55" t="s">
-        <v>83</v>
+        <v>167</v>
       </c>
       <c r="D55" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E55" t="s">
-        <v>197</v>
-      </c>
-      <c r="F55" t="s">
-        <v>202</v>
+        <v>227</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B56" t="s">
-        <v>147</v>
+        <v>195</v>
       </c>
       <c r="C56" t="s">
-        <v>84</v>
+        <v>168</v>
       </c>
       <c r="D56" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E56" t="s">
-        <v>196</v>
-      </c>
-      <c r="F56" t="s">
-        <v>202</v>
+        <v>228</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B57" t="s">
+        <v>196</v>
+      </c>
+      <c r="C57" t="s">
+        <v>169</v>
+      </c>
+      <c r="D57" t="s">
+        <v>211</v>
+      </c>
+      <c r="E57" t="s">
+        <v>142</v>
+      </c>
+      <c r="F57" t="s">
         <v>148</v>
-      </c>
-      <c r="C57" t="s">
-        <v>85</v>
-      </c>
-      <c r="D57" t="s">
-        <v>208</v>
-      </c>
-      <c r="E57" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B58" t="s">
-        <v>149</v>
+        <v>197</v>
       </c>
       <c r="C58" t="s">
-        <v>86</v>
+        <v>170</v>
       </c>
       <c r="D58" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E58" t="s">
-        <v>198</v>
+        <v>229</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B59" t="s">
-        <v>150</v>
+        <v>111</v>
       </c>
       <c r="C59" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="D59" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E59" t="s">
-        <v>160</v>
+        <v>230</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B60" t="s">
-        <v>151</v>
+        <v>112</v>
       </c>
       <c r="C60" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="D60" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E60" t="s">
-        <v>163</v>
+        <v>231</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B61" t="s">
-        <v>139</v>
+        <v>198</v>
       </c>
       <c r="C61" t="s">
-        <v>51</v>
+        <v>171</v>
       </c>
       <c r="D61" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E61" t="s">
-        <v>195</v>
+        <v>226</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B62" t="s">
-        <v>138</v>
+        <v>199</v>
       </c>
       <c r="C62" t="s">
-        <v>77</v>
+        <v>172</v>
       </c>
       <c r="D62" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E62" t="s">
-        <v>189</v>
-      </c>
-      <c r="F62" t="s">
-        <v>200</v>
+        <v>227</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B63" t="s">
-        <v>137</v>
+        <v>210</v>
       </c>
       <c r="C63" t="s">
-        <v>76</v>
+        <v>173</v>
       </c>
       <c r="D63" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E63" t="s">
-        <v>194</v>
+        <v>232</v>
       </c>
       <c r="F63" t="s">
-        <v>200</v>
+        <v>149</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B64" t="s">
-        <v>136</v>
+        <v>200</v>
       </c>
       <c r="C64" t="s">
-        <v>75</v>
+        <v>174</v>
       </c>
       <c r="D64" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E64" t="s">
-        <v>193</v>
+        <v>232</v>
+      </c>
+      <c r="F64" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B65" t="s">
-        <v>140</v>
+        <v>201</v>
       </c>
       <c r="C65" t="s">
-        <v>47</v>
+        <v>175</v>
       </c>
       <c r="D65" t="s">
-        <v>48</v>
+        <v>211</v>
       </c>
       <c r="E65" t="s">
-        <v>212</v>
+        <v>232</v>
+      </c>
+      <c r="F65" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B66" t="s">
-        <v>152</v>
+        <v>202</v>
       </c>
       <c r="C66" t="s">
-        <v>89</v>
+        <v>176</v>
       </c>
       <c r="D66" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E66" t="s">
-        <v>196</v>
+        <v>233</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B67" t="s">
-        <v>153</v>
+        <v>203</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>177</v>
       </c>
       <c r="D67" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E67" t="s">
-        <v>196</v>
+        <v>234</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B68" t="s">
-        <v>154</v>
+        <v>204</v>
       </c>
       <c r="C68" t="s">
-        <v>92</v>
+        <v>178</v>
       </c>
       <c r="D68" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E68" t="s">
-        <v>164</v>
-      </c>
-      <c r="F68" t="s">
-        <v>200</v>
+        <v>235</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B69" t="s">
-        <v>155</v>
+        <v>205</v>
       </c>
       <c r="C69" t="s">
-        <v>93</v>
+        <v>179</v>
       </c>
       <c r="D69" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E69" t="s">
-        <v>165</v>
-      </c>
-      <c r="F69" t="s">
-        <v>200</v>
+        <v>235</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B70" t="s">
-        <v>156</v>
+        <v>206</v>
       </c>
       <c r="C70" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="D70" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E70" t="s">
-        <v>196</v>
+        <v>236</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B71" t="s">
-        <v>157</v>
+        <v>207</v>
       </c>
       <c r="C71" t="s">
-        <v>91</v>
+        <v>181</v>
       </c>
       <c r="D71" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E71" t="s">
-        <v>196</v>
+        <v>237</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B72" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
       <c r="C72" t="s">
-        <v>76</v>
+        <v>182</v>
       </c>
       <c r="D72" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E72" t="s">
-        <v>194</v>
-      </c>
-      <c r="F72" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B73" t="s">
-        <v>138</v>
+        <v>209</v>
       </c>
       <c r="C73" t="s">
-        <v>77</v>
+        <v>183</v>
       </c>
       <c r="D73" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E73" t="s">
-        <v>189</v>
-      </c>
-      <c r="F73" t="s">
-        <v>200</v>
+        <v>226</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B74" t="s">
-        <v>136</v>
+        <v>109</v>
       </c>
       <c r="C74" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D74" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E74" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>49</v>
-      </c>
-      <c r="B75" t="s">
-        <v>139</v>
-      </c>
-      <c r="C75" t="s">
-        <v>51</v>
-      </c>
-      <c r="D75" t="s">
-        <v>208</v>
-      </c>
-      <c r="E75" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>49</v>
-      </c>
-      <c r="B76" t="s">
-        <v>140</v>
-      </c>
-      <c r="C76" t="s">
-        <v>47</v>
-      </c>
-      <c r="D76" t="s">
-        <v>48</v>
-      </c>
-      <c r="E76" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{756C4BFB-69BA-4E37-8A39-249423B4BF8F}">
+      <formula1>$I$3:$I$8</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2415,7 +2458,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E403C15-C2F0-4BBD-B389-CAB985F75BC2}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -2424,122 +2467,116 @@
     <col min="4" max="4" width="27.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>31</v>
       </c>
       <c r="B1" t="s">
-        <v>209</v>
+        <v>154</v>
       </c>
       <c r="C1" t="s">
-        <v>211</v>
+        <v>156</v>
       </c>
       <c r="D1" t="s">
-        <v>210</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
       <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B4" t="s">
         <v>35</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>35</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>203</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s">
         <v>37</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
         <v>37</v>
       </c>
-      <c r="D4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>45</v>
       </c>
-      <c r="B5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="B7" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>46</v>
       </c>
-      <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>41</v>
       </c>
-      <c r="C7" t="s">
-        <v>204</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D8" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" t="s">
-        <v>205</v>
-      </c>
-      <c r="D8" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
# Bugfixes for Dashboard # Klimsta Abschluss project export
</commit_message>
<xml_diff>
--- a/notebooks/Dashboard/chart_info.xlsx
+++ b/notebooks/Dashboard/chart_info.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ma1066\Documents\Code\peexcel\notebooks\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62ECC837-5829-4F19-AF29-300610FE0187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD95936-8309-4608-A9B1-DD77037F0F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{8863A408-E089-4CD0-AD5E-01FA994FFACD}"/>
+    <workbookView xWindow="4245" yWindow="4245" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{8863A408-E089-4CD0-AD5E-01FA994FFACD}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
     <sheet name="diagram_info" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="271">
   <si>
     <t>domain</t>
   </si>
@@ -165,12 +165,6 @@
     <t>build_four_column_gwp_chart</t>
   </si>
   <si>
-    <t>Multi-District Overview</t>
-  </si>
-  <si>
-    <t>build_multi_grid_chart</t>
-  </si>
-  <si>
     <t>gwp_ee</t>
   </si>
   <si>
@@ -180,9 +174,6 @@
     <t>district_gwp_ee</t>
   </si>
   <si>
-    <t>multi_chart</t>
-  </si>
-  <si>
     <t>EUI_plugAuxLight</t>
   </si>
   <si>
@@ -498,9 +489,6 @@
     <t>District GWP Breakdown (4-Column View)</t>
   </si>
   <si>
-    <t>District Comparision</t>
-  </si>
-  <si>
     <t>WW E-Stab</t>
   </si>
   <si>
@@ -754,19 +742,183 @@
   </si>
   <si>
     <t>#b87500</t>
+  </si>
+  <si>
+    <t>GWP_oe_lc_mob_export</t>
+  </si>
+  <si>
+    <t>GWP_oe_lc_mob_ev</t>
+  </si>
+  <si>
+    <t>GWP_oe_lc_mob_fossile</t>
+  </si>
+  <si>
+    <t>GWP_oe_lc_emission_savings</t>
+  </si>
+  <si>
+    <t>GWP_oe_lc_emission</t>
+  </si>
+  <si>
+    <t>GWP_ee_total_construction_biogenic</t>
+  </si>
+  <si>
+    <t>GWP_ee_lc_mob</t>
+  </si>
+  <si>
+    <t>GWP_ee_total_TES</t>
+  </si>
+  <si>
+    <t>GWP_ee_total_construction</t>
+  </si>
+  <si>
+    <t>GWP_lc_EE_total</t>
+  </si>
+  <si>
+    <t>GWP_lc_total</t>
+  </si>
+  <si>
+    <t>LV Mobilitäts-Export</t>
+  </si>
+  <si>
+    <t>LCA OE MIV elektrisch</t>
+  </si>
+  <si>
+    <t>LCA OE MIV fossil</t>
+  </si>
+  <si>
+    <t>LZ Betrieb Gebäude Vermiedene Emissionen</t>
+  </si>
+  <si>
+    <t>LZ Betrieb Gebäude Emissionen</t>
+  </si>
+  <si>
+    <t>THG Graue Energie LZ Baulich Biogen</t>
+  </si>
+  <si>
+    <t>Errichtung Mobilität</t>
+  </si>
+  <si>
+    <t>THG Graue Energie LZ TGA</t>
+  </si>
+  <si>
+    <t>THG Graue Energie LZ Baulich</t>
+  </si>
+  <si>
+    <t>EE THG-Emissionen 2025-2075</t>
+  </si>
+  <si>
+    <t>THG-Emissionen 2025-2075</t>
+  </si>
+  <si>
+    <t>#e9fd0e</t>
+  </si>
+  <si>
+    <t>#ffffc8</t>
+  </si>
+  <si>
+    <t>#b47602</t>
+  </si>
+  <si>
+    <t>#60b564</t>
+  </si>
+  <si>
+    <t>#951052</t>
+  </si>
+  <si>
+    <t>#f59c00</t>
+  </si>
+  <si>
+    <t>#eb4197</t>
+  </si>
+  <si>
+    <t>#1c575f</t>
+  </si>
+  <si>
+    <t>#33abba</t>
+  </si>
+  <si>
+    <t>#bbce00</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>y_axis_title</t>
+  </si>
+  <si>
+    <t>Primärenergie kWh/m²NGFa</t>
+  </si>
+  <si>
+    <t>kWh/m²NGFa</t>
+  </si>
+  <si>
+    <r>
+      <t>THG-Bilanz 2025-2075 (kg</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>CO2equiv.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>/m²</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>BGF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1126,9 +1278,45 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="8">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{689C6868-F4CC-41DD-81A9-29460501981F}">
+  <we:reference id="wa200006518" version="1.1.1.0" store="de-DE" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200006518" version="1.1.1.0" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="pyscriptSettings" value="&quot;{\&quot;defaultMode\&quot;:2,\&quot;pyodideVersion\&quot;:\&quot;0.26.2\&quot;,\&quot;pyodidePackages\&quot;:[\&quot;numpy\&quot;,\&quot;pandas\&quot;,\&quot;matplotlib\&quot;,\&quot;statsmodels\&quot;],\&quot;pyscriptApps\&quot;:[],\&quot;micropipPackages\&quot;:[\&quot;seaborn==0.13.2\&quot;],\&quot;initCode\&quot;:\&quot;# Add imports\\nimport math\\nimport numpy as np\\nimport pandas as pd\\n\\n# Define classes and functions\\ndef to_df(data) -&gt; pd.DataFrame:\\n    \\\&quot;\\\&quot;\\\&quot;\\n    Converts a REF (i.e. list of lists) into a pandas DataFrame\\n    Assumes that the first row contains column headers\\n\\n    Usage: df = to_df(REF(\\\&quot;F15:H22\\\&quot;))\\n    \\\&quot;\\\&quot;\\\&quot;\\n    if isinstance(data, pd.DataFrame):\\n        return data\\n    if hasattr(data, '__len__') and len(data) &gt; 0 and hasattr(data[0], '__len__'):\\n        return pd.DataFrame(data[1:], columns=data[0])\\n    raise TypeError('Expected list of lists')\\n\\ndef to_array(data) -&gt; np.ndarray:\\n    \\\&quot;\\\&quot;\\\&quot;\\n    Converts a REF (i.e. list of lists) into a 2-dimensional numpy array\\n\\n    Usage: arr = to_array(REF(\\\&quot;B3:C44\\\&quot;))\\n    \\\&quot;\\\&quot;\\\&quot;\\n    if isinstance(data, np.ndarray):\\n        return data\\n    return np.array(data)\\n\\ndef to_list(data) -&gt; list:\\n    \\\&quot;\\\&quot;\\\&quot;\\n    Converts a REF (i.e. list of lists) into a 1-d list.\\n    Handles wide (1xn) or tall (nx1) data.\\n\\n    Usage: x = to_list(REF(\\\&quot;G1:G55\\\&quot;))\\n    \\\&quot;\\\&quot;\\\&quot;\\n    if not hasattr(data, '__len__'): # data is scalar\\n        return [data]\\n    if len(data) == 0 or not hasattr(data[0], '__len__'): # data is already a list\\n        return list(data)\\n    if len(data) == 1: # data is wide\\n        return list(data[0])\\n    elif len(data[0]) == 1: #data is tall\\n        return [x[0] for x in data]\\n    else:\\n        raise TypeError(f\\\&quot;data must be 1xn or nx1, not {len(data)}x{len(data[0])}\\\&quot;)\\n\\n\&quot;}&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_PYSCRIPT_CODE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_ANACONDA_CODE</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{0858819E-0033-43BF-8937-05EC82904868}">
+      <we:backgroundApp state="0" runtimeId="PyScript.Url"/>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7A2313-314F-4C5D-9E95-F307104932AD}">
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -1161,7 +1349,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -1170,10 +1358,10 @@
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I2" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1181,7 +1369,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
@@ -1190,7 +1378,7 @@
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I3" t="s">
         <v>16</v>
@@ -1201,7 +1389,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -1210,7 +1398,7 @@
         <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I4" t="s">
         <v>17</v>
@@ -1221,7 +1409,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
@@ -1230,10 +1418,10 @@
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I5" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1241,7 +1429,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -1250,10 +1438,10 @@
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I6" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1261,7 +1449,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1270,10 +1458,10 @@
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1281,7 +1469,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
         <v>13</v>
@@ -1290,10 +1478,10 @@
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I8" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1301,7 +1489,7 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
@@ -1310,7 +1498,7 @@
         <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1318,7 +1506,7 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
@@ -1327,10 +1515,10 @@
         <v>16</v>
       </c>
       <c r="E10" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1338,7 +1526,7 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
@@ -1347,10 +1535,10 @@
         <v>17</v>
       </c>
       <c r="E11" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F11" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1358,7 +1546,7 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
@@ -1367,7 +1555,7 @@
         <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1375,7 +1563,7 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C13" t="s">
         <v>19</v>
@@ -1384,7 +1572,7 @@
         <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1392,7 +1580,7 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
@@ -1401,10 +1589,10 @@
         <v>17</v>
       </c>
       <c r="E14" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F14" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1412,7 +1600,7 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C15" t="s">
         <v>22</v>
@@ -1421,10 +1609,10 @@
         <v>17</v>
       </c>
       <c r="E15" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F15" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1432,7 +1620,7 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
         <v>24</v>
@@ -1441,7 +1629,7 @@
         <v>16</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1449,7 +1637,7 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
         <v>25</v>
@@ -1458,7 +1646,7 @@
         <v>16</v>
       </c>
       <c r="E17" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1466,7 +1654,7 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
         <v>26</v>
@@ -1475,7 +1663,7 @@
         <v>16</v>
       </c>
       <c r="E18" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1483,7 +1671,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
         <v>27</v>
@@ -1492,7 +1680,7 @@
         <v>16</v>
       </c>
       <c r="E19" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1500,7 +1688,7 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
         <v>28</v>
@@ -1509,7 +1697,7 @@
         <v>17</v>
       </c>
       <c r="E20" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1517,7 +1705,7 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C21" t="s">
         <v>29</v>
@@ -1526,7 +1714,7 @@
         <v>17</v>
       </c>
       <c r="E21" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1534,7 +1722,7 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
         <v>30</v>
@@ -1543,910 +1731,1296 @@
         <v>17</v>
       </c>
       <c r="E22" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B23" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D23" t="s">
         <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B24" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
         <v>16</v>
       </c>
       <c r="E24" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B25" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
         <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B26" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D26" t="s">
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B27" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D27" t="s">
         <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B29" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D29" t="s">
         <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C30" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D30" t="s">
         <v>17</v>
       </c>
       <c r="E30" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D31" t="s">
         <v>17</v>
       </c>
       <c r="E31" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B32" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C32" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
       </c>
       <c r="E32" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B33" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C33" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
       </c>
       <c r="E33" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C34" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D34" t="s">
         <v>17</v>
       </c>
       <c r="E34" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B35" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
       </c>
       <c r="E35" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C36" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D36" t="s">
         <v>17</v>
       </c>
       <c r="E36" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F36" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B37" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C37" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D37" t="s">
         <v>17</v>
       </c>
       <c r="E37" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B38" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C38" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
       </c>
       <c r="E38" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B39" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C39" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D39" t="s">
         <v>17</v>
       </c>
       <c r="E39" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>110</v>
+        <v>245</v>
       </c>
       <c r="C40" t="s">
-        <v>65</v>
+        <v>234</v>
       </c>
       <c r="D40" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E40" t="s">
-        <v>216</v>
+        <v>256</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B41" t="s">
-        <v>113</v>
+        <v>246</v>
       </c>
       <c r="C41" t="s">
-        <v>68</v>
+        <v>235</v>
       </c>
       <c r="D41" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E41" t="s">
-        <v>217</v>
+        <v>257</v>
+      </c>
+      <c r="F41" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>114</v>
+        <v>247</v>
       </c>
       <c r="C42" t="s">
-        <v>69</v>
+        <v>236</v>
       </c>
       <c r="D42" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E42" t="s">
-        <v>217</v>
+        <v>258</v>
+      </c>
+      <c r="F42" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>184</v>
+        <v>248</v>
       </c>
       <c r="C43" t="s">
-        <v>157</v>
+        <v>237</v>
       </c>
       <c r="D43" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E43" t="s">
-        <v>218</v>
+        <v>259</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B44" t="s">
-        <v>116</v>
+        <v>249</v>
       </c>
       <c r="C44" t="s">
-        <v>71</v>
+        <v>238</v>
       </c>
       <c r="D44" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E44" t="s">
-        <v>219</v>
+        <v>260</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B45" t="s">
-        <v>185</v>
+        <v>250</v>
       </c>
       <c r="C45" t="s">
-        <v>158</v>
+        <v>239</v>
       </c>
       <c r="D45" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E45" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B46" t="s">
-        <v>186</v>
+        <v>251</v>
       </c>
       <c r="C46" t="s">
-        <v>159</v>
+        <v>240</v>
       </c>
       <c r="D46" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E46" t="s">
-        <v>219</v>
+        <v>261</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B47" t="s">
-        <v>115</v>
+        <v>252</v>
       </c>
       <c r="C47" t="s">
-        <v>70</v>
+        <v>241</v>
       </c>
       <c r="D47" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E47" t="s">
-        <v>218</v>
+        <v>262</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B48" t="s">
+        <v>253</v>
+      </c>
+      <c r="C48" t="s">
+        <v>242</v>
+      </c>
+      <c r="D48" t="s">
+        <v>207</v>
+      </c>
+      <c r="E48" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>41</v>
+      </c>
+      <c r="B49" t="s">
+        <v>254</v>
+      </c>
+      <c r="C49" t="s">
+        <v>243</v>
+      </c>
+      <c r="D49" t="s">
+        <v>209</v>
+      </c>
+      <c r="E49" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>41</v>
+      </c>
+      <c r="B50" t="s">
+        <v>255</v>
+      </c>
+      <c r="C50" t="s">
+        <v>244</v>
+      </c>
+      <c r="D50" t="s">
+        <v>210</v>
+      </c>
+      <c r="E50" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>42</v>
+      </c>
+      <c r="B51" t="s">
+        <v>107</v>
+      </c>
+      <c r="C51" t="s">
+        <v>62</v>
+      </c>
+      <c r="D51" t="s">
+        <v>207</v>
+      </c>
+      <c r="E51" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>42</v>
+      </c>
+      <c r="B52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" t="s">
+        <v>65</v>
+      </c>
+      <c r="D52" t="s">
+        <v>207</v>
+      </c>
+      <c r="E52" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>42</v>
+      </c>
+      <c r="B53" t="s">
+        <v>111</v>
+      </c>
+      <c r="C53" t="s">
+        <v>66</v>
+      </c>
+      <c r="D53" t="s">
+        <v>207</v>
+      </c>
+      <c r="E53" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>42</v>
+      </c>
+      <c r="B54" t="s">
+        <v>180</v>
+      </c>
+      <c r="C54" t="s">
+        <v>153</v>
+      </c>
+      <c r="D54" t="s">
+        <v>207</v>
+      </c>
+      <c r="E54" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>42</v>
+      </c>
+      <c r="B55" t="s">
+        <v>113</v>
+      </c>
+      <c r="C55" t="s">
+        <v>68</v>
+      </c>
+      <c r="D55" t="s">
+        <v>207</v>
+      </c>
+      <c r="E55" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>42</v>
+      </c>
+      <c r="B56" t="s">
+        <v>181</v>
+      </c>
+      <c r="C56" t="s">
+        <v>154</v>
+      </c>
+      <c r="D56" t="s">
+        <v>207</v>
+      </c>
+      <c r="E56" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>42</v>
+      </c>
+      <c r="B57" t="s">
+        <v>182</v>
+      </c>
+      <c r="C57" t="s">
+        <v>155</v>
+      </c>
+      <c r="D57" t="s">
+        <v>207</v>
+      </c>
+      <c r="E57" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58" t="s">
+        <v>112</v>
+      </c>
+      <c r="C58" t="s">
+        <v>67</v>
+      </c>
+      <c r="D58" t="s">
+        <v>207</v>
+      </c>
+      <c r="E58" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>42</v>
+      </c>
+      <c r="B59" t="s">
+        <v>183</v>
+      </c>
+      <c r="C59" t="s">
+        <v>156</v>
+      </c>
+      <c r="D59" t="s">
+        <v>207</v>
+      </c>
+      <c r="E59" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>42</v>
+      </c>
+      <c r="B60" t="s">
+        <v>184</v>
+      </c>
+      <c r="C60" t="s">
+        <v>157</v>
+      </c>
+      <c r="D60" t="s">
+        <v>207</v>
+      </c>
+      <c r="E60" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>42</v>
+      </c>
+      <c r="B61" t="s">
+        <v>185</v>
+      </c>
+      <c r="C61" t="s">
+        <v>158</v>
+      </c>
+      <c r="D61" t="s">
+        <v>207</v>
+      </c>
+      <c r="E61" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>42</v>
+      </c>
+      <c r="B62" t="s">
+        <v>186</v>
+      </c>
+      <c r="C62" t="s">
+        <v>159</v>
+      </c>
+      <c r="D62" t="s">
+        <v>207</v>
+      </c>
+      <c r="E62" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>42</v>
+      </c>
+      <c r="B63" t="s">
         <v>187</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C63" t="s">
         <v>160</v>
       </c>
-      <c r="D48" t="s">
-        <v>211</v>
-      </c>
-      <c r="E48" t="s">
+      <c r="D63" t="s">
+        <v>207</v>
+      </c>
+      <c r="E63" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>44</v>
-      </c>
-      <c r="B49" t="s">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>42</v>
+      </c>
+      <c r="B64" t="s">
         <v>188</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C64" t="s">
         <v>161</v>
       </c>
-      <c r="D49" t="s">
-        <v>211</v>
-      </c>
-      <c r="E49" t="s">
+      <c r="D64" t="s">
+        <v>207</v>
+      </c>
+      <c r="E64" t="s">
         <v>221</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B50" t="s">
-        <v>189</v>
-      </c>
-      <c r="C50" t="s">
-        <v>162</v>
-      </c>
-      <c r="D50" t="s">
-        <v>211</v>
-      </c>
-      <c r="E50" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>44</v>
-      </c>
-      <c r="B51" t="s">
-        <v>190</v>
-      </c>
-      <c r="C51" t="s">
-        <v>163</v>
-      </c>
-      <c r="D51" t="s">
-        <v>211</v>
-      </c>
-      <c r="E51" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>44</v>
-      </c>
-      <c r="B52" t="s">
-        <v>191</v>
-      </c>
-      <c r="C52" t="s">
-        <v>164</v>
-      </c>
-      <c r="D52" t="s">
-        <v>211</v>
-      </c>
-      <c r="E52" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>44</v>
-      </c>
-      <c r="B53" t="s">
-        <v>192</v>
-      </c>
-      <c r="C53" t="s">
-        <v>165</v>
-      </c>
-      <c r="D53" t="s">
-        <v>211</v>
-      </c>
-      <c r="E53" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>44</v>
-      </c>
-      <c r="B54" t="s">
-        <v>193</v>
-      </c>
-      <c r="C54" t="s">
-        <v>166</v>
-      </c>
-      <c r="D54" t="s">
-        <v>211</v>
-      </c>
-      <c r="E54" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>44</v>
-      </c>
-      <c r="B55" t="s">
-        <v>194</v>
-      </c>
-      <c r="C55" t="s">
-        <v>167</v>
-      </c>
-      <c r="D55" t="s">
-        <v>211</v>
-      </c>
-      <c r="E55" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>44</v>
-      </c>
-      <c r="B56" t="s">
-        <v>195</v>
-      </c>
-      <c r="C56" t="s">
-        <v>168</v>
-      </c>
-      <c r="D56" t="s">
-        <v>211</v>
-      </c>
-      <c r="E56" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>44</v>
-      </c>
-      <c r="B57" t="s">
-        <v>196</v>
-      </c>
-      <c r="C57" t="s">
-        <v>169</v>
-      </c>
-      <c r="D57" t="s">
-        <v>211</v>
-      </c>
-      <c r="E57" t="s">
-        <v>142</v>
-      </c>
-      <c r="F57" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>44</v>
-      </c>
-      <c r="B58" t="s">
-        <v>197</v>
-      </c>
-      <c r="C58" t="s">
-        <v>170</v>
-      </c>
-      <c r="D58" t="s">
-        <v>211</v>
-      </c>
-      <c r="E58" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>44</v>
-      </c>
-      <c r="B59" t="s">
-        <v>111</v>
-      </c>
-      <c r="C59" t="s">
-        <v>66</v>
-      </c>
-      <c r="D59" t="s">
-        <v>211</v>
-      </c>
-      <c r="E59" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>44</v>
-      </c>
-      <c r="B60" t="s">
-        <v>112</v>
-      </c>
-      <c r="C60" t="s">
-        <v>67</v>
-      </c>
-      <c r="D60" t="s">
-        <v>211</v>
-      </c>
-      <c r="E60" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>44</v>
-      </c>
-      <c r="B61" t="s">
-        <v>198</v>
-      </c>
-      <c r="C61" t="s">
-        <v>171</v>
-      </c>
-      <c r="D61" t="s">
-        <v>211</v>
-      </c>
-      <c r="E61" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>44</v>
-      </c>
-      <c r="B62" t="s">
-        <v>199</v>
-      </c>
-      <c r="C62" t="s">
-        <v>172</v>
-      </c>
-      <c r="D62" t="s">
-        <v>211</v>
-      </c>
-      <c r="E62" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>44</v>
-      </c>
-      <c r="B63" t="s">
-        <v>210</v>
-      </c>
-      <c r="C63" t="s">
-        <v>173</v>
-      </c>
-      <c r="D63" t="s">
-        <v>211</v>
-      </c>
-      <c r="E63" t="s">
-        <v>232</v>
-      </c>
-      <c r="F63" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>44</v>
-      </c>
-      <c r="B64" t="s">
-        <v>200</v>
-      </c>
-      <c r="C64" t="s">
-        <v>174</v>
-      </c>
-      <c r="D64" t="s">
-        <v>211</v>
-      </c>
-      <c r="E64" t="s">
-        <v>232</v>
-      </c>
-      <c r="F64" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B65" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C65" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="D65" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E65" t="s">
-        <v>232</v>
-      </c>
-      <c r="F65" t="s">
-        <v>149</v>
+        <v>222</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B66" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="C66" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D66" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E66" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B67" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="C67" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="D67" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E67" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B68" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="C68" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="D68" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E68" t="s">
-        <v>235</v>
+        <v>139</v>
+      </c>
+      <c r="F68" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B69" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="C69" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="D69" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E69" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B70" t="s">
-        <v>206</v>
+        <v>108</v>
       </c>
       <c r="C70" t="s">
-        <v>180</v>
+        <v>63</v>
       </c>
       <c r="D70" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E70" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B71" t="s">
-        <v>207</v>
+        <v>109</v>
       </c>
       <c r="C71" t="s">
-        <v>181</v>
+        <v>64</v>
       </c>
       <c r="D71" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E71" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B72" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="C72" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="D72" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E72" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B73" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="C73" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="D73" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E73" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B74" t="s">
-        <v>109</v>
+        <v>206</v>
       </c>
       <c r="C74" t="s">
-        <v>64</v>
+        <v>169</v>
       </c>
       <c r="D74" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E74" t="s">
-        <v>226</v>
+        <v>228</v>
+      </c>
+      <c r="F74" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>42</v>
+      </c>
+      <c r="B75" t="s">
+        <v>196</v>
+      </c>
+      <c r="C75" t="s">
+        <v>170</v>
+      </c>
+      <c r="D75" t="s">
+        <v>207</v>
+      </c>
+      <c r="E75" t="s">
+        <v>228</v>
+      </c>
+      <c r="F75" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>42</v>
+      </c>
+      <c r="B76" t="s">
+        <v>197</v>
+      </c>
+      <c r="C76" t="s">
+        <v>171</v>
+      </c>
+      <c r="D76" t="s">
+        <v>207</v>
+      </c>
+      <c r="E76" t="s">
+        <v>228</v>
+      </c>
+      <c r="F76" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>42</v>
+      </c>
+      <c r="B77" t="s">
+        <v>198</v>
+      </c>
+      <c r="C77" t="s">
+        <v>172</v>
+      </c>
+      <c r="D77" t="s">
+        <v>207</v>
+      </c>
+      <c r="E77" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>42</v>
+      </c>
+      <c r="B78" t="s">
+        <v>199</v>
+      </c>
+      <c r="C78" t="s">
+        <v>173</v>
+      </c>
+      <c r="D78" t="s">
+        <v>207</v>
+      </c>
+      <c r="E78" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>42</v>
+      </c>
+      <c r="B79" t="s">
+        <v>200</v>
+      </c>
+      <c r="C79" t="s">
+        <v>174</v>
+      </c>
+      <c r="D79" t="s">
+        <v>207</v>
+      </c>
+      <c r="E79" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>42</v>
+      </c>
+      <c r="B80" t="s">
+        <v>201</v>
+      </c>
+      <c r="C80" t="s">
+        <v>175</v>
+      </c>
+      <c r="D80" t="s">
+        <v>207</v>
+      </c>
+      <c r="E80" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>42</v>
+      </c>
+      <c r="B81" t="s">
+        <v>202</v>
+      </c>
+      <c r="C81" t="s">
+        <v>176</v>
+      </c>
+      <c r="D81" t="s">
+        <v>207</v>
+      </c>
+      <c r="E81" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>42</v>
+      </c>
+      <c r="B82" t="s">
+        <v>203</v>
+      </c>
+      <c r="C82" t="s">
+        <v>177</v>
+      </c>
+      <c r="D82" t="s">
+        <v>207</v>
+      </c>
+      <c r="E82" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>42</v>
+      </c>
+      <c r="B83" t="s">
+        <v>204</v>
+      </c>
+      <c r="C83" t="s">
+        <v>178</v>
+      </c>
+      <c r="D83" t="s">
+        <v>207</v>
+      </c>
+      <c r="E83" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>42</v>
+      </c>
+      <c r="B84" t="s">
+        <v>205</v>
+      </c>
+      <c r="C84" t="s">
+        <v>179</v>
+      </c>
+      <c r="D84" t="s">
+        <v>207</v>
+      </c>
+      <c r="E84" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>42</v>
+      </c>
+      <c r="B85" t="s">
+        <v>106</v>
+      </c>
+      <c r="C85" t="s">
+        <v>61</v>
+      </c>
+      <c r="D85" t="s">
+        <v>207</v>
+      </c>
+      <c r="E85" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>43</v>
+      </c>
+      <c r="B86" t="s">
+        <v>245</v>
+      </c>
+      <c r="C86" t="s">
+        <v>234</v>
+      </c>
+      <c r="D86" t="s">
+        <v>210</v>
+      </c>
+      <c r="E86" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>43</v>
+      </c>
+      <c r="B87" t="s">
+        <v>246</v>
+      </c>
+      <c r="C87" t="s">
+        <v>235</v>
+      </c>
+      <c r="D87" t="s">
+        <v>208</v>
+      </c>
+      <c r="E87" t="s">
+        <v>257</v>
+      </c>
+      <c r="F87" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>43</v>
+      </c>
+      <c r="B88" t="s">
+        <v>247</v>
+      </c>
+      <c r="C88" t="s">
+        <v>236</v>
+      </c>
+      <c r="D88" t="s">
+        <v>208</v>
+      </c>
+      <c r="E88" t="s">
+        <v>258</v>
+      </c>
+      <c r="F88" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>43</v>
+      </c>
+      <c r="B89" t="s">
+        <v>248</v>
+      </c>
+      <c r="C89" t="s">
+        <v>237</v>
+      </c>
+      <c r="D89" t="s">
+        <v>210</v>
+      </c>
+      <c r="E89" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>43</v>
+      </c>
+      <c r="B90" t="s">
+        <v>249</v>
+      </c>
+      <c r="C90" t="s">
+        <v>238</v>
+      </c>
+      <c r="D90" t="s">
+        <v>208</v>
+      </c>
+      <c r="E90" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>43</v>
+      </c>
+      <c r="B91" t="s">
+        <v>250</v>
+      </c>
+      <c r="C91" t="s">
+        <v>239</v>
+      </c>
+      <c r="D91" t="s">
+        <v>209</v>
+      </c>
+      <c r="E91" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>43</v>
+      </c>
+      <c r="B92" t="s">
+        <v>251</v>
+      </c>
+      <c r="C92" t="s">
+        <v>240</v>
+      </c>
+      <c r="D92" t="s">
+        <v>207</v>
+      </c>
+      <c r="E92" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>43</v>
+      </c>
+      <c r="B93" t="s">
+        <v>252</v>
+      </c>
+      <c r="C93" t="s">
+        <v>241</v>
+      </c>
+      <c r="D93" t="s">
+        <v>207</v>
+      </c>
+      <c r="E93" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>43</v>
+      </c>
+      <c r="B94" t="s">
+        <v>253</v>
+      </c>
+      <c r="C94" t="s">
+        <v>242</v>
+      </c>
+      <c r="D94" t="s">
+        <v>207</v>
+      </c>
+      <c r="E94" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>43</v>
+      </c>
+      <c r="B95" t="s">
+        <v>254</v>
+      </c>
+      <c r="C95" t="s">
+        <v>243</v>
+      </c>
+      <c r="D95" t="s">
+        <v>209</v>
+      </c>
+      <c r="E95" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>43</v>
+      </c>
+      <c r="B96" t="s">
+        <v>255</v>
+      </c>
+      <c r="C96" t="s">
+        <v>244</v>
+      </c>
+      <c r="D96" t="s">
+        <v>210</v>
+      </c>
+      <c r="E96" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{756C4BFB-69BA-4E37-8A39-249423B4BF8F}">
       <formula1>$I$3:$I$8</formula1>
     </dataValidation>
@@ -2458,30 +3032,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E403C15-C2F0-4BBD-B389-CAB985F75BC2}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.5703125" customWidth="1"/>
     <col min="4" max="4" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>31</v>
       </c>
       <c r="B1" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C1" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+      <c r="E1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2494,8 +3072,11 @@
       <c r="D2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -2508,10 +3089,13 @@
       <c r="D3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
@@ -2522,10 +3106,13 @@
       <c r="D4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="18.75" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
         <v>36</v>
@@ -2536,47 +3123,42 @@
       <c r="D5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="18.75" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="18.75" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D7" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>152</v>
-      </c>
-      <c r="D8" t="s">
-        <v>42</v>
+      <c r="E7" t="s">
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>